<commit_message>
updated grouping of metabolites on diverging bars
</commit_message>
<xml_diff>
--- a/Databases/QC/manual_QC_repo.xlsx
+++ b/Databases/QC/manual_QC_repo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdp2019/Desktop/PGD-postop-metabolomics/Databases/QC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{943F7384-C0D7-3B4B-831F-F3798FE64110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E5EA3A-C2C0-7D43-9E43-557915946659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="22560" windowHeight="17720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="curated_spec" sheetId="16" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="422">
   <si>
     <t>Identified_Name</t>
   </si>
@@ -1240,9 +1240,6 @@
     <t>Cellular Energetics</t>
   </si>
   <si>
-    <t>Inflammation</t>
-  </si>
-  <si>
     <t>Redox</t>
   </si>
   <si>
@@ -1306,10 +1303,10 @@
     <t>N-Glycolylglucosamine</t>
   </si>
   <si>
-    <t>Vascular Signaling</t>
-  </si>
-  <si>
     <t>Ap5A</t>
+  </si>
+  <si>
+    <t>Immunometabolic Signaling</t>
   </si>
 </sst>
 </file>
@@ -1988,56 +1985,58 @@
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>217</v>
+        <v>41</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="C3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>360</v>
+        <v>331</v>
       </c>
       <c r="G3" s="12">
-        <v>1.779746875546653</v>
+        <v>-0.44325155465499583</v>
       </c>
       <c r="H3" s="12">
-        <v>3.4638840419138168E-5</v>
+        <v>0.1353118509221457</v>
       </c>
       <c r="I3" s="12">
-        <v>-0.47542374833514067</v>
+        <v>0.78892055215644774</v>
       </c>
       <c r="J3" s="12">
-        <v>0.63892167026263857</v>
+        <v>1.9671208112267899E-2</v>
       </c>
       <c r="K3" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>338</v>
-      </c>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
+        <v>305</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>24</v>
+      </c>
       <c r="P3" s="5" t="s">
         <v>23</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="R3" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>219</v>
-      </c>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
       <c r="T3" s="2" t="s">
-        <v>220</v>
+        <v>42</v>
       </c>
       <c r="U3" s="2"/>
       <c r="V3" s="2" t="s">
@@ -2047,16 +2046,16 @@
         <v>23</v>
       </c>
       <c r="X3" s="2">
-        <v>335.09500000000003</v>
+        <v>344.27957600000002</v>
       </c>
       <c r="Y3" s="2">
-        <v>183</v>
+        <v>57.995856000000003</v>
       </c>
       <c r="Z3" s="2" t="s">
-        <v>141</v>
+        <v>28</v>
       </c>
       <c r="AA3" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AB3" s="2" t="s">
         <v>23</v>
@@ -2066,56 +2065,58 @@
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="11" t="s">
-        <v>421</v>
+      <c r="D4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>398</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="G4" s="12">
-        <v>-0.21232771886722551</v>
+        <v>1.4296981753017159</v>
       </c>
       <c r="H4" s="12">
-        <v>3.2347958530699238E-2</v>
+        <v>3.8902343919267942E-3</v>
       </c>
       <c r="I4" s="12">
-        <v>6.2649205201758207E-2</v>
+        <v>1.563555661607094</v>
       </c>
       <c r="J4" s="12">
-        <v>0.56166950064806109</v>
+        <v>1.990833078500114E-3</v>
       </c>
       <c r="K4" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
       <c r="P4" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>23</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="U4" s="2"/>
       <c r="V4" s="2" t="s">
@@ -2125,10 +2126,10 @@
         <v>23</v>
       </c>
       <c r="X4" s="2">
-        <v>242.06989999999999</v>
+        <v>175.0248</v>
       </c>
       <c r="Y4" s="2">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="Z4" s="2" t="s">
         <v>40</v>
@@ -2144,38 +2145,40 @@
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C5" s="2"/>
+        <v>155</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>361</v>
+        <v>331</v>
       </c>
       <c r="G5" s="12">
-        <v>0.24141717347866631</v>
+        <v>0.70088283571846688</v>
       </c>
       <c r="H5" s="12">
-        <v>0.55280427491186623</v>
+        <v>3.0454582706448751E-2</v>
       </c>
       <c r="I5" s="12">
-        <v>2.0707014376494581</v>
+        <v>0.83570289737371084</v>
       </c>
       <c r="J5" s="12">
-        <v>1.7532161293423039E-3</v>
+        <v>2.9397095112831308E-2</v>
       </c>
       <c r="K5" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
@@ -2186,12 +2189,10 @@
       <c r="Q5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="R5" s="2" t="s">
-        <v>135</v>
-      </c>
+      <c r="R5" s="2"/>
       <c r="S5" s="2"/>
       <c r="T5" s="2" t="s">
-        <v>136</v>
+        <v>204</v>
       </c>
       <c r="U5" s="2"/>
       <c r="V5" s="2" t="s">
@@ -2201,13 +2202,13 @@
         <v>23</v>
       </c>
       <c r="X5" s="2">
-        <v>407.20750099999998</v>
+        <v>246.169984</v>
       </c>
       <c r="Y5" s="2">
-        <v>153.490116</v>
+        <v>87.6</v>
       </c>
       <c r="Z5" s="2" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="AA5" s="2" t="s">
         <v>25</v>
@@ -2220,12 +2221,14 @@
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="2"/>
+        <v>372</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
@@ -2233,45 +2236,43 @@
         <v>398</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>331</v>
+        <v>354</v>
       </c>
       <c r="G6" s="12">
-        <v>-0.44325155465499583</v>
+        <v>1.543116915257126</v>
       </c>
       <c r="H6" s="12">
-        <v>0.1353118509221457</v>
+        <v>1.2526678136343301E-4</v>
       </c>
       <c r="I6" s="12">
-        <v>0.78892055215644774</v>
+        <v>1.204485873455001</v>
       </c>
       <c r="J6" s="12">
-        <v>1.9671208112267899E-2</v>
+        <v>1.1309822990967341E-4</v>
       </c>
       <c r="K6" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>305</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>307</v>
+      </c>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
       <c r="P6" s="5" t="s">
         <v>23</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
+      <c r="R6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>52</v>
+      </c>
       <c r="T6" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="U6" s="2"/>
       <c r="V6" s="2" t="s">
@@ -2281,16 +2282,16 @@
         <v>23</v>
       </c>
       <c r="X6" s="2">
-        <v>344.27957600000002</v>
+        <v>131.08269999999999</v>
       </c>
       <c r="Y6" s="2">
-        <v>57.995856000000003</v>
+        <v>51</v>
       </c>
       <c r="Z6" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AB6" s="2" t="s">
         <v>23</v>
@@ -2300,40 +2301,38 @@
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>63</v>
+        <v>190</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="11" t="s">
         <v>398</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>353</v>
+      <c r="F7" s="11" t="s">
+        <v>331</v>
       </c>
       <c r="G7" s="12">
-        <v>1.4296981753017159</v>
+        <v>0.42774598695724819</v>
       </c>
       <c r="H7" s="12">
-        <v>3.8902343919267942E-3</v>
+        <v>0.1753351233680619</v>
       </c>
       <c r="I7" s="12">
-        <v>1.563555661607094</v>
+        <v>1.1007596474091981</v>
       </c>
       <c r="J7" s="12">
-        <v>1.990833078500114E-3</v>
+        <v>4.2028322357151324E-3</v>
       </c>
       <c r="K7" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
@@ -2345,49 +2344,47 @@
         <v>23</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>65</v>
-      </c>
+        <v>191</v>
+      </c>
+      <c r="S7" s="2"/>
       <c r="T7" s="2" t="s">
-        <v>66</v>
+        <v>192</v>
       </c>
       <c r="U7" s="2"/>
       <c r="V7" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W7" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X7" s="2">
-        <v>175.0248</v>
+        <v>232.15433400000001</v>
       </c>
       <c r="Y7" s="2">
-        <v>144</v>
+        <v>95.3</v>
       </c>
       <c r="Z7" s="2" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="AA7" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AB7" s="2" t="s">
         <v>23</v>
       </c>
       <c r="AC7" s="2"/>
-      <c r="AD7" s="2"/>
+      <c r="AD7" s="2" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>155</v>
+        <v>213</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>394</v>
+      </c>
+      <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
@@ -2398,22 +2395,22 @@
         <v>331</v>
       </c>
       <c r="G8" s="12">
-        <v>0.70088283571846688</v>
+        <v>0.30961790936737899</v>
       </c>
       <c r="H8" s="12">
-        <v>3.0454582706448751E-2</v>
+        <v>0.31061866603254817</v>
       </c>
       <c r="I8" s="12">
-        <v>0.83570289737371084</v>
+        <v>1.1223761667074541</v>
       </c>
       <c r="J8" s="12">
-        <v>2.9397095112831308E-2</v>
+        <v>2.2457589986286121E-3</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
@@ -2424,10 +2421,12 @@
       <c r="Q8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="R8" s="2"/>
+      <c r="R8" s="2" t="s">
+        <v>214</v>
+      </c>
       <c r="S8" s="2"/>
       <c r="T8" s="2" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="U8" s="2"/>
       <c r="V8" s="2" t="s">
@@ -2437,10 +2436,10 @@
         <v>23</v>
       </c>
       <c r="X8" s="2">
-        <v>246.169984</v>
+        <v>288.21693399999998</v>
       </c>
       <c r="Y8" s="2">
-        <v>87.6</v>
+        <v>70.2</v>
       </c>
       <c r="Z8" s="2" t="s">
         <v>28</v>
@@ -2449,21 +2448,21 @@
         <v>25</v>
       </c>
       <c r="AB8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AC8" s="2"/>
+        <v>24</v>
+      </c>
+      <c r="AC8" s="2" t="s">
+        <v>216</v>
+      </c>
       <c r="AD8" s="2"/>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>151</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>389</v>
+      </c>
+      <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
@@ -2474,22 +2473,22 @@
         <v>354</v>
       </c>
       <c r="G9" s="12">
-        <v>1.543116915257126</v>
+        <v>-0.2203761482568645</v>
       </c>
       <c r="H9" s="12">
-        <v>1.2526678136343301E-4</v>
+        <v>0.52396947932538485</v>
       </c>
       <c r="I9" s="12">
-        <v>1.204485873455001</v>
+        <v>0.74925893154757617</v>
       </c>
       <c r="J9" s="12">
-        <v>1.1309822990967341E-4</v>
+        <v>2.369458388956398E-2</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>307</v>
+        <v>330</v>
       </c>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
@@ -2501,13 +2500,13 @@
         <v>23</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>51</v>
+        <v>152</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>52</v>
+        <v>153</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>53</v>
+        <v>154</v>
       </c>
       <c r="U9" s="2"/>
       <c r="V9" s="2" t="s">
@@ -2517,13 +2516,13 @@
         <v>23</v>
       </c>
       <c r="X9" s="2">
-        <v>131.08269999999999</v>
+        <v>131.01599999999999</v>
       </c>
       <c r="Y9" s="2">
-        <v>51</v>
+        <v>215</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="AA9" s="2" t="s">
         <v>29</v>
@@ -2536,40 +2535,38 @@
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>143</v>
+        <v>182</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>390</v>
+      </c>
+      <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>363</v>
+        <v>354</v>
       </c>
       <c r="G10" s="12">
-        <v>0.48424095268319078</v>
+        <v>5.7765515545963098E-2</v>
       </c>
       <c r="H10" s="12">
-        <v>2.0953495472482059E-2</v>
+        <v>0.83265392194610122</v>
       </c>
       <c r="I10" s="12">
-        <v>0.32629335681689042</v>
+        <v>0.62615101076087498</v>
       </c>
       <c r="J10" s="12">
-        <v>4.5943350323316499E-2</v>
+        <v>6.842428840644393E-5</v>
       </c>
       <c r="K10" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
@@ -2581,13 +2578,11 @@
         <v>23</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="S10" s="2" t="s">
-        <v>145</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="S10" s="2"/>
       <c r="T10" s="2" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
       <c r="U10" s="2"/>
       <c r="V10" s="2" t="s">
@@ -2597,10 +2592,10 @@
         <v>23</v>
       </c>
       <c r="X10" s="2">
-        <v>118.0652</v>
+        <v>204.08680000000001</v>
       </c>
       <c r="Y10" s="2">
-        <v>151</v>
+        <v>279</v>
       </c>
       <c r="Z10" s="2" t="s">
         <v>28</v>
@@ -2616,40 +2611,38 @@
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>395</v>
+      </c>
+      <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>362</v>
+        <v>331</v>
       </c>
       <c r="G11" s="12">
-        <v>1.1679592301085471</v>
+        <v>0.16181307824404101</v>
       </c>
       <c r="H11" s="12">
-        <v>3.04141659440837E-2</v>
+        <v>0.7447526411269817</v>
       </c>
       <c r="I11" s="12">
-        <v>1.3982873055507239</v>
+        <v>1.5336865152561681</v>
       </c>
       <c r="J11" s="12">
-        <v>3.305475126456589E-2</v>
+        <v>3.5616451135334383E-2</v>
       </c>
       <c r="K11" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>
@@ -2661,13 +2654,13 @@
         <v>23</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="U11" s="2"/>
       <c r="V11" s="2" t="s">
@@ -2677,13 +2670,13 @@
         <v>23</v>
       </c>
       <c r="X11" s="2">
-        <v>263.10329999999999</v>
+        <v>284.11180000000002</v>
       </c>
       <c r="Y11" s="2">
-        <v>58</v>
+        <v>188</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="AA11" s="2" t="s">
         <v>29</v>
@@ -2696,40 +2689,38 @@
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>369</v>
+        <v>354</v>
       </c>
       <c r="G12" s="12">
-        <v>0.63355426504666212</v>
+        <v>-7.2827907266004743E-2</v>
       </c>
       <c r="H12" s="12">
-        <v>6.8428999046584629E-2</v>
+        <v>0.95534208495987971</v>
       </c>
       <c r="I12" s="12">
-        <v>0.60184795892662635</v>
+        <v>1.913044615838313</v>
       </c>
       <c r="J12" s="12">
-        <v>4.3256641483210401E-2</v>
+        <v>1.716324160172484E-3</v>
       </c>
       <c r="K12" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
@@ -2741,13 +2732,11 @@
         <v>23</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="S12" s="2" t="s">
-        <v>163</v>
-      </c>
+        <v>170</v>
+      </c>
+      <c r="S12" s="2"/>
       <c r="T12" s="2" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="U12" s="2"/>
       <c r="V12" s="2" t="s">
@@ -2757,16 +2746,16 @@
         <v>23</v>
       </c>
       <c r="X12" s="2">
-        <v>161.03790000000001</v>
+        <v>174.050164</v>
       </c>
       <c r="Y12" s="2">
-        <v>171</v>
+        <v>169.9359</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="AA12" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AB12" s="2" t="s">
         <v>23</v>
@@ -2776,40 +2765,38 @@
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>107</v>
+        <v>188</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>358</v>
+      <c r="E13" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>331</v>
       </c>
       <c r="G13" s="12">
-        <v>0.92703432152064735</v>
+        <v>0.30766258225711951</v>
       </c>
       <c r="H13" s="12">
-        <v>2.7251602861135978E-2</v>
+        <v>0.31843591296621598</v>
       </c>
       <c r="I13" s="12">
-        <v>0.94820046279419579</v>
+        <v>1.1137629052321361</v>
       </c>
       <c r="J13" s="12">
-        <v>1.244681915664534E-2</v>
+        <v>1.0030988581828311E-2</v>
       </c>
       <c r="K13" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
@@ -2821,13 +2808,11 @@
         <v>23</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>109</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="S13" s="2"/>
       <c r="T13" s="2" t="s">
-        <v>110</v>
+        <v>189</v>
       </c>
       <c r="U13" s="2"/>
       <c r="V13" s="2" t="s">
@@ -2837,16 +2822,16 @@
         <v>23</v>
       </c>
       <c r="X13" s="2">
-        <v>333.04930000000002</v>
+        <v>218.13868400000001</v>
       </c>
       <c r="Y13" s="2">
-        <v>149</v>
+        <v>108.4</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="AA13" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AB13" s="2" t="s">
         <v>23</v>
@@ -2856,38 +2841,38 @@
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>190</v>
+        <v>119</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>190</v>
+        <v>119</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>331</v>
+      <c r="F14" s="2" t="s">
+        <v>356</v>
       </c>
       <c r="G14" s="12">
-        <v>0.42774598695724819</v>
+        <v>-1.8687288582560409E-2</v>
       </c>
       <c r="H14" s="12">
-        <v>0.1753351233680619</v>
+        <v>0.96148439384437845</v>
       </c>
       <c r="I14" s="12">
-        <v>1.1007596474091981</v>
+        <v>-0.44872313389006457</v>
       </c>
       <c r="J14" s="12">
-        <v>4.2028322357151324E-3</v>
+        <v>4.2645217558800387E-2</v>
       </c>
       <c r="K14" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
@@ -2899,27 +2884,27 @@
         <v>23</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>191</v>
+        <v>120</v>
       </c>
       <c r="S14" s="2"/>
       <c r="T14" s="2" t="s">
-        <v>192</v>
+        <v>121</v>
       </c>
       <c r="U14" s="2"/>
       <c r="V14" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="X14" s="2">
-        <v>232.15433400000001</v>
+        <v>375.13102400000002</v>
       </c>
       <c r="Y14" s="2">
-        <v>95.3</v>
+        <v>136.169016</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="AA14" s="2" t="s">
         <v>25</v>
@@ -2928,16 +2913,14 @@
         <v>23</v>
       </c>
       <c r="AC14" s="2"/>
-      <c r="AD14" s="2" t="s">
-        <v>193</v>
-      </c>
+      <c r="AD14" s="2"/>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>394</v>
+        <v>233</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2" t="s">
@@ -2950,22 +2933,22 @@
         <v>331</v>
       </c>
       <c r="G15" s="12">
-        <v>0.30961790936737899</v>
+        <v>-0.23932679806917179</v>
       </c>
       <c r="H15" s="12">
-        <v>0.31061866603254817</v>
+        <v>0.49324288642045638</v>
       </c>
       <c r="I15" s="12">
-        <v>1.1223761667074541</v>
+        <v>0.6928158058499605</v>
       </c>
       <c r="J15" s="12">
-        <v>2.2457589986286121E-3</v>
+        <v>4.2852870485354508E-2</v>
       </c>
       <c r="K15" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="M15" s="7"/>
       <c r="N15" s="7"/>
@@ -2976,12 +2959,10 @@
       <c r="Q15" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="R15" s="2" t="s">
-        <v>214</v>
-      </c>
+      <c r="R15" s="2"/>
       <c r="S15" s="2"/>
       <c r="T15" s="2" t="s">
-        <v>215</v>
+        <v>234</v>
       </c>
       <c r="U15" s="2"/>
       <c r="V15" s="2" t="s">
@@ -2991,10 +2972,10 @@
         <v>23</v>
       </c>
       <c r="X15" s="2">
-        <v>288.21693399999998</v>
+        <v>372.310835</v>
       </c>
       <c r="Y15" s="2">
-        <v>70.2</v>
+        <v>62.8</v>
       </c>
       <c r="Z15" s="2" t="s">
         <v>28</v>
@@ -3003,47 +2984,45 @@
         <v>25</v>
       </c>
       <c r="AB15" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AC15" s="2" t="s">
-        <v>216</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="AC15" s="2"/>
       <c r="AD15" s="2"/>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>151</v>
+        <v>111</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
         <v>398</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G16" s="12">
-        <v>-0.2203761482568645</v>
+        <v>1.8935577572401081</v>
       </c>
       <c r="H16" s="12">
-        <v>0.52396947932538485</v>
+        <v>1.194906365241895E-3</v>
       </c>
       <c r="I16" s="12">
-        <v>0.74925893154757617</v>
+        <v>0.2088079376948038</v>
       </c>
       <c r="J16" s="12">
-        <v>2.369458388956398E-2</v>
+        <v>0.87770009349523637</v>
       </c>
       <c r="K16" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="M16" s="7"/>
       <c r="N16" s="7"/>
@@ -3055,13 +3034,13 @@
         <v>23</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>152</v>
+        <v>112</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>153</v>
+        <v>113</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2" t="s">
@@ -3071,13 +3050,13 @@
         <v>23</v>
       </c>
       <c r="X16" s="2">
-        <v>131.01599999999999</v>
+        <v>357.10430000000002</v>
       </c>
       <c r="Y16" s="2">
-        <v>215</v>
+        <v>56</v>
       </c>
       <c r="Z16" s="2" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="AA16" s="2" t="s">
         <v>29</v>
@@ -3090,15 +3069,15 @@
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>182</v>
+        <v>243</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
         <v>398</v>
       </c>
@@ -3106,22 +3085,22 @@
         <v>354</v>
       </c>
       <c r="G17" s="12">
-        <v>5.7765515545963098E-2</v>
+        <v>0.33202077710400962</v>
       </c>
       <c r="H17" s="12">
-        <v>0.83265392194610122</v>
+        <v>8.0086262192070642E-2</v>
       </c>
       <c r="I17" s="12">
-        <v>0.62615101076087498</v>
+        <v>0.61102624684128415</v>
       </c>
       <c r="J17" s="12">
-        <v>6.842428840644393E-5</v>
+        <v>1.962899894050529E-2</v>
       </c>
       <c r="K17" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
@@ -3133,11 +3112,13 @@
         <v>23</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="S17" s="2"/>
+        <v>244</v>
+      </c>
+      <c r="S17" s="2" t="s">
+        <v>245</v>
+      </c>
       <c r="T17" s="2" t="s">
-        <v>184</v>
+        <v>246</v>
       </c>
       <c r="U17" s="2"/>
       <c r="V17" s="2" t="s">
@@ -3147,10 +3128,10 @@
         <v>23</v>
       </c>
       <c r="X17" s="2">
-        <v>204.08680000000001</v>
+        <v>90.055000000000007</v>
       </c>
       <c r="Y17" s="2">
-        <v>279</v>
+        <v>179</v>
       </c>
       <c r="Z17" s="2" t="s">
         <v>28</v>
@@ -3166,38 +3147,38 @@
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>103</v>
+        <v>200</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
         <v>398</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>331</v>
+        <v>356</v>
       </c>
       <c r="G18" s="12">
-        <v>0.16181307824404101</v>
+        <v>0.84761372576020655</v>
       </c>
       <c r="H18" s="12">
-        <v>0.7447526411269817</v>
+        <v>1.168905677663227E-2</v>
       </c>
       <c r="I18" s="12">
-        <v>1.5336865152561681</v>
+        <v>0.52434557560937911</v>
       </c>
       <c r="J18" s="12">
-        <v>3.5616451135334383E-2</v>
+        <v>7.3173614173116255E-2</v>
       </c>
       <c r="K18" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>318</v>
+        <v>344</v>
       </c>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
@@ -3209,13 +3190,13 @@
         <v>23</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>104</v>
+        <v>201</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>105</v>
+        <v>202</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>106</v>
+        <v>203</v>
       </c>
       <c r="U18" s="2"/>
       <c r="V18" s="2" t="s">
@@ -3225,13 +3206,13 @@
         <v>23</v>
       </c>
       <c r="X18" s="2">
-        <v>284.11180000000002</v>
+        <v>245.095</v>
       </c>
       <c r="Y18" s="2">
-        <v>188</v>
+        <v>94</v>
       </c>
       <c r="Z18" s="2" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="AA18" s="2" t="s">
         <v>29</v>
@@ -3244,38 +3225,38 @@
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>169</v>
+        <v>239</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
         <v>398</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="G19" s="12">
-        <v>-7.2827907266004743E-2</v>
+        <v>1.3484735218485771</v>
       </c>
       <c r="H19" s="12">
-        <v>0.95534208495987971</v>
+        <v>1.2450651528625499E-3</v>
       </c>
       <c r="I19" s="12">
-        <v>1.913044615838313</v>
+        <v>0.57720537269963401</v>
       </c>
       <c r="J19" s="12">
-        <v>1.716324160172484E-3</v>
+        <v>0.48299480934489808</v>
       </c>
       <c r="K19" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>336</v>
+        <v>352</v>
       </c>
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
@@ -3287,11 +3268,13 @@
         <v>23</v>
       </c>
       <c r="R19" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="S19" s="2"/>
+        <v>240</v>
+      </c>
+      <c r="S19" s="2" t="s">
+        <v>241</v>
+      </c>
       <c r="T19" s="2" t="s">
-        <v>171</v>
+        <v>242</v>
       </c>
       <c r="U19" s="2"/>
       <c r="V19" s="2" t="s">
@@ -3301,16 +3284,16 @@
         <v>23</v>
       </c>
       <c r="X19" s="2">
-        <v>174.050164</v>
+        <v>769.13879999999995</v>
       </c>
       <c r="Y19" s="2">
-        <v>169.9359</v>
+        <v>99</v>
       </c>
       <c r="Z19" s="2" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="AA19" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AB19" s="2" t="s">
         <v>23</v>
@@ -3320,38 +3303,38 @@
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>188</v>
+        <v>55</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="D20" s="2"/>
+      <c r="E20" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="F20" s="11" t="s">
-        <v>331</v>
+      <c r="F20" s="2" t="s">
+        <v>354</v>
       </c>
       <c r="G20" s="12">
-        <v>0.30766258225711951</v>
+        <v>0.53221524900362027</v>
       </c>
       <c r="H20" s="12">
-        <v>0.31843591296621598</v>
+        <v>8.8651383189041529E-3</v>
       </c>
       <c r="I20" s="12">
-        <v>1.1137629052321361</v>
+        <v>0.17387178526495009</v>
       </c>
       <c r="J20" s="12">
-        <v>1.0030988581828311E-2</v>
+        <v>0.46311227870137539</v>
       </c>
       <c r="K20" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
@@ -3363,11 +3346,13 @@
         <v>23</v>
       </c>
       <c r="R20" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="S20" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="S20" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="T20" s="2" t="s">
-        <v>189</v>
+        <v>58</v>
       </c>
       <c r="U20" s="2"/>
       <c r="V20" s="2" t="s">
@@ -3377,16 +3362,16 @@
         <v>23</v>
       </c>
       <c r="X20" s="2">
-        <v>218.13868400000001</v>
+        <v>145.06190000000001</v>
       </c>
       <c r="Y20" s="2">
-        <v>108.4</v>
+        <v>49</v>
       </c>
       <c r="Z20" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="AA20" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AB20" s="2" t="s">
         <v>23</v>
@@ -3396,38 +3381,38 @@
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>119</v>
+        <v>194</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D21" s="2"/>
       <c r="E21" s="2" t="s">
         <v>398</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="G21" s="12">
-        <v>-1.8687288582560409E-2</v>
+        <v>-0.34209170609178591</v>
       </c>
       <c r="H21" s="12">
-        <v>0.96148439384437845</v>
+        <v>4.0685975658821011E-2</v>
       </c>
       <c r="I21" s="12">
-        <v>-0.44872313389006457</v>
+        <v>9.2526691120513149E-2</v>
       </c>
       <c r="J21" s="12">
-        <v>4.2645217558800387E-2</v>
+        <v>0.66402733718679485</v>
       </c>
       <c r="K21" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>322</v>
+        <v>342</v>
       </c>
       <c r="M21" s="7"/>
       <c r="N21" s="7"/>
@@ -3439,11 +3424,13 @@
         <v>23</v>
       </c>
       <c r="R21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="S21" s="2"/>
+        <v>195</v>
+      </c>
+      <c r="S21" s="2" t="s">
+        <v>196</v>
+      </c>
       <c r="T21" s="2" t="s">
-        <v>121</v>
+        <v>197</v>
       </c>
       <c r="U21" s="2"/>
       <c r="V21" s="2" t="s">
@@ -3453,16 +3440,16 @@
         <v>23</v>
       </c>
       <c r="X21" s="2">
-        <v>375.13102400000002</v>
+        <v>236.9992</v>
       </c>
       <c r="Y21" s="2">
-        <v>136.169016</v>
+        <v>152</v>
       </c>
       <c r="Z21" s="2" t="s">
-        <v>35</v>
+        <v>141</v>
       </c>
       <c r="AA21" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AB21" s="2" t="s">
         <v>23</v>
@@ -3472,38 +3459,38 @@
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>233</v>
+        <v>26</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="D22" s="2"/>
+      <c r="E22" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="F22" s="11" t="s">
-        <v>331</v>
+      <c r="F22" s="2" t="s">
+        <v>354</v>
       </c>
       <c r="G22" s="12">
-        <v>-0.23932679806917179</v>
+        <v>0.36028887884359762</v>
       </c>
       <c r="H22" s="12">
-        <v>0.49324288642045638</v>
+        <v>1.532998388181952E-2</v>
       </c>
       <c r="I22" s="12">
-        <v>0.6928158058499605</v>
+        <v>0.29408265831335001</v>
       </c>
       <c r="J22" s="12">
-        <v>4.2852870485354508E-2</v>
+        <v>0.1097603211429076</v>
       </c>
       <c r="K22" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="M22" s="7"/>
       <c r="N22" s="7"/>
@@ -3514,10 +3501,14 @@
       <c r="Q22" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="R22" s="2"/>
-      <c r="S22" s="2"/>
+      <c r="R22" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="S22" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="T22" s="2" t="s">
-        <v>234</v>
+        <v>62</v>
       </c>
       <c r="U22" s="2"/>
       <c r="V22" s="2" t="s">
@@ -3527,16 +3518,16 @@
         <v>23</v>
       </c>
       <c r="X22" s="2">
-        <v>372.310835</v>
+        <v>164.0718</v>
       </c>
       <c r="Y22" s="2">
-        <v>62.8</v>
+        <v>58</v>
       </c>
       <c r="Z22" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="AA22" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AB22" s="2" t="s">
         <v>23</v>
@@ -3546,38 +3537,38 @@
     </row>
     <row r="23" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>75</v>
+        <v>165</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D23" s="2"/>
       <c r="E23" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>363</v>
+        <v>354</v>
       </c>
       <c r="G23" s="12">
-        <v>1.0301828711344569</v>
+        <v>0.31242018585406578</v>
       </c>
       <c r="H23" s="12">
-        <v>0.47108709263359339</v>
+        <v>3.34157587829343E-3</v>
       </c>
       <c r="I23" s="12">
-        <v>2.2529238052341221</v>
+        <v>4.794351271877062E-2</v>
       </c>
       <c r="J23" s="12">
-        <v>4.74205255360741E-2</v>
+        <v>0.78408739378422754</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L23" s="10" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="M23" s="7"/>
       <c r="N23" s="7"/>
@@ -3589,13 +3580,13 @@
         <v>23</v>
       </c>
       <c r="R23" s="2" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="S23" s="2" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="T23" s="2" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="U23" s="2"/>
       <c r="V23" s="2" t="s">
@@ -3605,10 +3596,10 @@
         <v>23</v>
       </c>
       <c r="X23" s="2">
-        <v>138.05500000000001</v>
+        <v>165.05459999999999</v>
       </c>
       <c r="Y23" s="2">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="Z23" s="2" t="s">
         <v>28</v>
@@ -3624,38 +3615,38 @@
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D24" s="2"/>
       <c r="E24" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="G24" s="12">
-        <v>0.28175063782081372</v>
+        <v>0.74213009626279813</v>
       </c>
       <c r="H24" s="12">
-        <v>0.24980479836988309</v>
+        <v>7.0743312657492357E-3</v>
       </c>
       <c r="I24" s="12">
-        <v>0.44978955218162753</v>
+        <v>-0.20339225141119319</v>
       </c>
       <c r="J24" s="12">
-        <v>3.9871676963873347E-3</v>
+        <v>0.65523178463825249</v>
       </c>
       <c r="K24" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L24" s="10" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="M24" s="7"/>
       <c r="N24" s="7"/>
@@ -3667,13 +3658,11 @@
         <v>23</v>
       </c>
       <c r="R24" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="S24" s="2" t="s">
-        <v>48</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="S24" s="2"/>
       <c r="T24" s="2" t="s">
-        <v>49</v>
+        <v>85</v>
       </c>
       <c r="U24" s="2"/>
       <c r="V24" s="2" t="s">
@@ -3683,10 +3672,10 @@
         <v>23</v>
       </c>
       <c r="X24" s="2">
-        <v>129.01939999999999</v>
+        <v>229.01230000000001</v>
       </c>
       <c r="Y24" s="2">
-        <v>55</v>
+        <v>199</v>
       </c>
       <c r="Z24" s="2" t="s">
         <v>35</v>
@@ -3702,38 +3691,38 @@
     </row>
     <row r="25" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>185</v>
+        <v>122</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D25" s="2"/>
       <c r="E25" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="G25" s="12">
-        <v>0.49998172242149508</v>
+        <v>0.58223576143027067</v>
       </c>
       <c r="H25" s="12">
-        <v>2.3309906065451791E-4</v>
+        <v>4.2694027106335783E-2</v>
       </c>
       <c r="I25" s="12">
-        <v>0.17614573135977449</v>
+        <v>0.39619576717556088</v>
       </c>
       <c r="J25" s="12">
-        <v>0.16391224111632141</v>
+        <v>0.28127257421310192</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L25" s="10" t="s">
-        <v>341</v>
+        <v>323</v>
       </c>
       <c r="M25" s="7"/>
       <c r="N25" s="7"/>
@@ -3745,11 +3734,13 @@
         <v>23</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="S25" s="2"/>
+        <v>123</v>
+      </c>
+      <c r="S25" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="T25" s="2" t="s">
-        <v>187</v>
+        <v>125</v>
       </c>
       <c r="U25" s="2"/>
       <c r="V25" s="2" t="s">
@@ -3759,13 +3750,13 @@
         <v>23</v>
       </c>
       <c r="X25" s="2">
-        <v>213.14850000000001</v>
+        <v>379.03930000000003</v>
       </c>
       <c r="Y25" s="2">
-        <v>105</v>
+        <v>147</v>
       </c>
       <c r="Z25" s="2" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="AA25" s="2" t="s">
         <v>29</v>
@@ -3778,38 +3769,38 @@
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>367</v>
+        <v>354</v>
       </c>
       <c r="G26" s="12">
-        <v>0.55019015312911712</v>
+        <v>0.40997998758135168</v>
       </c>
       <c r="H26" s="12">
-        <v>0.62756353499656081</v>
+        <v>5.8644107209904336E-3</v>
       </c>
       <c r="I26" s="12">
-        <v>1.9264605376319219</v>
+        <v>0.27764180048433929</v>
       </c>
       <c r="J26" s="12">
-        <v>9.8541326104743202E-3</v>
+        <v>0.26137876946803812</v>
       </c>
       <c r="K26" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L26" s="10" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="M26" s="7"/>
       <c r="N26" s="7"/>
@@ -3821,11 +3812,13 @@
         <v>23</v>
       </c>
       <c r="R26" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="S26" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="S26" s="2" t="s">
+        <v>73</v>
+      </c>
       <c r="T26" s="2" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="U26" s="2"/>
       <c r="V26" s="2" t="s">
@@ -3835,13 +3828,13 @@
         <v>23</v>
       </c>
       <c r="X26" s="2">
-        <v>262.06950000000001</v>
+        <v>180.06659999999999</v>
       </c>
       <c r="Y26" s="2">
-        <v>134</v>
+        <v>58</v>
       </c>
       <c r="Z26" s="2" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="AA26" s="2" t="s">
         <v>29</v>
@@ -3854,48 +3847,44 @@
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>36</v>
+        <v>143</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C27" s="2"/>
+        <v>143</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D27" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>400</v>
+        <v>421</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="G27" s="12">
-        <v>0.41550808127715649</v>
+        <v>0.48424095268319078</v>
       </c>
       <c r="H27" s="12">
-        <v>0.42507349571591369</v>
+        <v>2.0953495472482059E-2</v>
       </c>
       <c r="I27" s="12">
-        <v>1.256760204695194</v>
+        <v>0.32629335681689042</v>
       </c>
       <c r="J27" s="12">
-        <v>4.4252755026857682E-3</v>
+        <v>4.5943350323316499E-2</v>
       </c>
       <c r="K27" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L27" s="10" t="s">
-        <v>304</v>
-      </c>
-      <c r="M27" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="N27" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="O27" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>328</v>
+      </c>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
       <c r="P27" s="5" t="s">
         <v>23</v>
       </c>
@@ -3903,13 +3892,13 @@
         <v>23</v>
       </c>
       <c r="R27" s="2" t="s">
-        <v>37</v>
+        <v>144</v>
       </c>
       <c r="S27" s="2" t="s">
-        <v>38</v>
+        <v>145</v>
       </c>
       <c r="T27" s="2" t="s">
-        <v>39</v>
+        <v>146</v>
       </c>
       <c r="U27" s="2"/>
       <c r="V27" s="2" t="s">
@@ -3919,13 +3908,13 @@
         <v>23</v>
       </c>
       <c r="X27" s="2">
-        <v>89.024500000000003</v>
+        <v>118.0652</v>
       </c>
       <c r="Y27" s="2">
-        <v>180</v>
+        <v>151</v>
       </c>
       <c r="Z27" s="2" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="AA27" s="2" t="s">
         <v>29</v>
@@ -3938,38 +3927,40 @@
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>206</v>
+        <v>96</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C28" s="2"/>
+        <v>96</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D28" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>400</v>
+        <v>421</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="G28" s="12">
-        <v>0.81129313979982598</v>
+        <v>1.1679592301085471</v>
       </c>
       <c r="H28" s="12">
-        <v>0.39017026025005369</v>
+        <v>3.04141659440837E-2</v>
       </c>
       <c r="I28" s="12">
-        <v>1.4308769326288799</v>
+        <v>1.3982873055507239</v>
       </c>
       <c r="J28" s="12">
-        <v>4.0284930069031888E-2</v>
+        <v>3.305475126456589E-2</v>
       </c>
       <c r="K28" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L28" s="10" t="s">
-        <v>345</v>
+        <v>317</v>
       </c>
       <c r="M28" s="7"/>
       <c r="N28" s="7"/>
@@ -3981,11 +3972,13 @@
         <v>23</v>
       </c>
       <c r="R28" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="S28" s="2"/>
+        <v>97</v>
+      </c>
+      <c r="S28" s="2" t="s">
+        <v>98</v>
+      </c>
       <c r="T28" s="2" t="s">
-        <v>208</v>
+        <v>99</v>
       </c>
       <c r="U28" s="2"/>
       <c r="V28" s="2" t="s">
@@ -3995,13 +3988,13 @@
         <v>23</v>
       </c>
       <c r="X28" s="2">
-        <v>283.14440000000002</v>
+        <v>263.10329999999999</v>
       </c>
       <c r="Y28" s="2">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="Z28" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="AA28" s="2" t="s">
         <v>29</v>
@@ -4014,38 +4007,38 @@
     </row>
     <row r="29" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>147</v>
+        <v>75</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>147</v>
+        <v>75</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>400</v>
+        <v>421</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="G29" s="12">
-        <v>0.26808666413641552</v>
+        <v>1.0301828711344569</v>
       </c>
       <c r="H29" s="12">
-        <v>0.1217336748932811</v>
+        <v>0.47108709263359339</v>
       </c>
       <c r="I29" s="12">
-        <v>0.58286136999222293</v>
+        <v>2.2529238052341221</v>
       </c>
       <c r="J29" s="12">
-        <v>1.042644163461523E-2</v>
+        <v>4.74205255360741E-2</v>
       </c>
       <c r="K29" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L29" s="10" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="M29" s="7"/>
       <c r="N29" s="7"/>
@@ -4057,13 +4050,13 @@
         <v>23</v>
       </c>
       <c r="R29" s="2" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="S29" s="2" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="T29" s="2" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="U29" s="2"/>
       <c r="V29" s="2" t="s">
@@ -4073,10 +4066,10 @@
         <v>23</v>
       </c>
       <c r="X29" s="2">
-        <v>123.0552</v>
+        <v>138.05500000000001</v>
       </c>
       <c r="Y29" s="2">
-        <v>27</v>
+        <v>162</v>
       </c>
       <c r="Z29" s="2" t="s">
         <v>28</v>
@@ -4092,38 +4085,38 @@
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>115</v>
+        <v>46</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>393</v>
+        <v>46</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E30" s="11" t="s">
+      <c r="E30" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="F30" s="11" t="s">
-        <v>361</v>
+      <c r="F30" s="2" t="s">
+        <v>362</v>
       </c>
       <c r="G30" s="12">
-        <v>0.52082421505483723</v>
+        <v>0.28175063782081372</v>
       </c>
       <c r="H30" s="12">
-        <v>0.18143830225368149</v>
+        <v>0.24980479836988309</v>
       </c>
       <c r="I30" s="12">
-        <v>1.2338926633816949</v>
+        <v>0.44978955218162753</v>
       </c>
       <c r="J30" s="12">
-        <v>2.0195633925086439E-3</v>
+        <v>3.9871676963873347E-3</v>
       </c>
       <c r="K30" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L30" s="10" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
       <c r="M30" s="7"/>
       <c r="N30" s="7"/>
@@ -4135,13 +4128,13 @@
         <v>23</v>
       </c>
       <c r="R30" s="2" t="s">
-        <v>116</v>
+        <v>47</v>
       </c>
       <c r="S30" s="2" t="s">
-        <v>117</v>
+        <v>48</v>
       </c>
       <c r="T30" s="2" t="s">
-        <v>118</v>
+        <v>49</v>
       </c>
       <c r="U30" s="2"/>
       <c r="V30" s="2" t="s">
@@ -4151,10 +4144,10 @@
         <v>23</v>
       </c>
       <c r="X30" s="2">
-        <v>367.15780000000001</v>
+        <v>129.01939999999999</v>
       </c>
       <c r="Y30" s="2">
-        <v>148</v>
+        <v>55</v>
       </c>
       <c r="Z30" s="2" t="s">
         <v>35</v>
@@ -4170,38 +4163,38 @@
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>111</v>
+        <v>380</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
-        <v>398</v>
+        <v>421</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="G31" s="12">
-        <v>1.8935577572401081</v>
+        <v>0.78621412149081848</v>
       </c>
       <c r="H31" s="12">
-        <v>1.194906365241895E-3</v>
+        <v>1.3185947511990931E-2</v>
       </c>
       <c r="I31" s="12">
-        <v>0.2088079376948038</v>
+        <v>0.28763142206793191</v>
       </c>
       <c r="J31" s="12">
-        <v>0.87770009349523637</v>
+        <v>0.43716304463804939</v>
       </c>
       <c r="K31" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L31" s="10" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="M31" s="7"/>
       <c r="N31" s="7"/>
@@ -4213,13 +4206,11 @@
         <v>23</v>
       </c>
       <c r="R31" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="S31" s="2" t="s">
-        <v>113</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="S31" s="2"/>
       <c r="T31" s="2" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="U31" s="2"/>
       <c r="V31" s="2" t="s">
@@ -4229,10 +4220,10 @@
         <v>23</v>
       </c>
       <c r="X31" s="2">
-        <v>357.10430000000002</v>
+        <v>398.00619999999998</v>
       </c>
       <c r="Y31" s="2">
-        <v>56</v>
+        <v>138</v>
       </c>
       <c r="Z31" s="2" t="s">
         <v>40</v>
@@ -4248,38 +4239,38 @@
     </row>
     <row r="32" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>243</v>
+        <v>178</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>373</v>
+        <v>386</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2" t="s">
-        <v>398</v>
+        <v>421</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="G32" s="12">
-        <v>0.33202077710400962</v>
+        <v>0.53781869393490922</v>
       </c>
       <c r="H32" s="12">
-        <v>8.0086262192070642E-2</v>
+        <v>3.7055885051282877E-2</v>
       </c>
       <c r="I32" s="12">
-        <v>0.61102624684128415</v>
+        <v>0.13663548694990621</v>
       </c>
       <c r="J32" s="12">
-        <v>1.962899894050529E-2</v>
+        <v>0.55005347203021426</v>
       </c>
       <c r="K32" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L32" s="10" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="M32" s="7"/>
       <c r="N32" s="7"/>
@@ -4291,13 +4282,13 @@
         <v>23</v>
       </c>
       <c r="R32" s="2" t="s">
-        <v>244</v>
+        <v>179</v>
       </c>
       <c r="S32" s="2" t="s">
-        <v>245</v>
+        <v>180</v>
       </c>
       <c r="T32" s="2" t="s">
-        <v>246</v>
+        <v>181</v>
       </c>
       <c r="U32" s="2"/>
       <c r="V32" s="2" t="s">
@@ -4307,10 +4298,10 @@
         <v>23</v>
       </c>
       <c r="X32" s="2">
-        <v>90.055000000000007</v>
+        <v>198.0881</v>
       </c>
       <c r="Y32" s="2">
-        <v>179</v>
+        <v>59</v>
       </c>
       <c r="Z32" s="2" t="s">
         <v>28</v>
@@ -4326,38 +4317,38 @@
     </row>
     <row r="33" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>200</v>
+        <v>225</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>200</v>
+        <v>387</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2" t="s">
-        <v>398</v>
+        <v>421</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="G33" s="12">
-        <v>0.84761372576020655</v>
+        <v>1.449497195603316</v>
       </c>
       <c r="H33" s="12">
-        <v>1.168905677663227E-2</v>
+        <v>2.4084407570208119E-3</v>
       </c>
       <c r="I33" s="12">
-        <v>0.52434557560937911</v>
+        <v>0.52907850064326922</v>
       </c>
       <c r="J33" s="12">
-        <v>7.3173614173116255E-2</v>
+        <v>0.36733938692032359</v>
       </c>
       <c r="K33" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L33" s="10" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="M33" s="7"/>
       <c r="N33" s="7"/>
@@ -4369,13 +4360,11 @@
         <v>23</v>
       </c>
       <c r="R33" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="S33" s="2" t="s">
-        <v>202</v>
-      </c>
+        <v>226</v>
+      </c>
+      <c r="S33" s="2"/>
       <c r="T33" s="2" t="s">
-        <v>203</v>
+        <v>227</v>
       </c>
       <c r="U33" s="2"/>
       <c r="V33" s="2" t="s">
@@ -4385,16 +4374,16 @@
         <v>23</v>
       </c>
       <c r="X33" s="2">
-        <v>245.095</v>
+        <v>339.17747600000001</v>
       </c>
       <c r="Y33" s="2">
-        <v>94</v>
+        <v>204.30355800000001</v>
       </c>
       <c r="Z33" s="2" t="s">
-        <v>28</v>
+        <v>228</v>
       </c>
       <c r="AA33" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AB33" s="2" t="s">
         <v>23</v>
@@ -4404,38 +4393,40 @@
     </row>
     <row r="34" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>239</v>
+        <v>161</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>239</v>
+        <v>161</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D34" s="2"/>
+      <c r="D34" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="E34" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>356</v>
+        <v>369</v>
       </c>
       <c r="G34" s="12">
-        <v>1.3484735218485771</v>
+        <v>0.63355426504666212</v>
       </c>
       <c r="H34" s="12">
-        <v>1.2450651528625499E-3</v>
+        <v>6.8428999046584629E-2</v>
       </c>
       <c r="I34" s="12">
-        <v>0.57720537269963401</v>
+        <v>0.60184795892662635</v>
       </c>
       <c r="J34" s="12">
-        <v>0.48299480934489808</v>
+        <v>4.3256641483210401E-2</v>
       </c>
       <c r="K34" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L34" s="10" t="s">
-        <v>352</v>
+        <v>334</v>
       </c>
       <c r="M34" s="7"/>
       <c r="N34" s="7"/>
@@ -4447,13 +4438,13 @@
         <v>23</v>
       </c>
       <c r="R34" s="2" t="s">
-        <v>240</v>
+        <v>162</v>
       </c>
       <c r="S34" s="2" t="s">
-        <v>241</v>
+        <v>163</v>
       </c>
       <c r="T34" s="2" t="s">
-        <v>242</v>
+        <v>164</v>
       </c>
       <c r="U34" s="2"/>
       <c r="V34" s="2" t="s">
@@ -4463,13 +4454,13 @@
         <v>23</v>
       </c>
       <c r="X34" s="2">
-        <v>769.13879999999995</v>
+        <v>161.03790000000001</v>
       </c>
       <c r="Y34" s="2">
-        <v>99</v>
+        <v>171</v>
       </c>
       <c r="Z34" s="2" t="s">
-        <v>156</v>
+        <v>27</v>
       </c>
       <c r="AA34" s="2" t="s">
         <v>29</v>
@@ -4482,38 +4473,40 @@
     </row>
     <row r="35" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>55</v>
+        <v>107</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>374</v>
+        <v>383</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D35" s="2"/>
+      <c r="D35" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="E35" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="G35" s="12">
-        <v>0.53221524900362027</v>
+        <v>0.92703432152064735</v>
       </c>
       <c r="H35" s="12">
-        <v>8.8651383189041529E-3</v>
+        <v>2.7251602861135978E-2</v>
       </c>
       <c r="I35" s="12">
-        <v>0.17387178526495009</v>
+        <v>0.94820046279419579</v>
       </c>
       <c r="J35" s="12">
-        <v>0.46311227870137539</v>
+        <v>1.244681915664534E-2</v>
       </c>
       <c r="K35" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L35" s="10" t="s">
-        <v>308</v>
+        <v>319</v>
       </c>
       <c r="M35" s="7"/>
       <c r="N35" s="7"/>
@@ -4525,13 +4518,13 @@
         <v>23</v>
       </c>
       <c r="R35" s="2" t="s">
-        <v>56</v>
+        <v>108</v>
       </c>
       <c r="S35" s="2" t="s">
-        <v>57</v>
+        <v>109</v>
       </c>
       <c r="T35" s="2" t="s">
-        <v>58</v>
+        <v>110</v>
       </c>
       <c r="U35" s="2"/>
       <c r="V35" s="2" t="s">
@@ -4541,10 +4534,10 @@
         <v>23</v>
       </c>
       <c r="X35" s="2">
-        <v>145.06190000000001</v>
+        <v>333.04930000000002</v>
       </c>
       <c r="Y35" s="2">
-        <v>49</v>
+        <v>149</v>
       </c>
       <c r="Z35" s="2" t="s">
         <v>35</v>
@@ -4560,38 +4553,38 @@
     </row>
     <row r="36" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C36" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D36" s="2"/>
       <c r="E36" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="G36" s="12">
-        <v>-0.34209170609178591</v>
+        <v>0.49998172242149508</v>
       </c>
       <c r="H36" s="12">
-        <v>4.0685975658821011E-2</v>
+        <v>2.3309906065451791E-4</v>
       </c>
       <c r="I36" s="12">
-        <v>9.2526691120513149E-2</v>
+        <v>0.17614573135977449</v>
       </c>
       <c r="J36" s="12">
-        <v>0.66402733718679485</v>
+        <v>0.16391224111632141</v>
       </c>
       <c r="K36" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="M36" s="7"/>
       <c r="N36" s="7"/>
@@ -4603,13 +4596,11 @@
         <v>23</v>
       </c>
       <c r="R36" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="S36" s="2" t="s">
-        <v>196</v>
-      </c>
+        <v>186</v>
+      </c>
+      <c r="S36" s="2"/>
       <c r="T36" s="2" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="U36" s="2"/>
       <c r="V36" s="2" t="s">
@@ -4619,13 +4610,13 @@
         <v>23</v>
       </c>
       <c r="X36" s="2">
-        <v>236.9992</v>
+        <v>213.14850000000001</v>
       </c>
       <c r="Y36" s="2">
-        <v>152</v>
+        <v>105</v>
       </c>
       <c r="Z36" s="2" t="s">
-        <v>141</v>
+        <v>28</v>
       </c>
       <c r="AA36" s="2" t="s">
         <v>29</v>
@@ -4638,38 +4629,38 @@
     </row>
     <row r="37" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>26</v>
+        <v>93</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="C37" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="G37" s="12">
-        <v>0.36028887884359762</v>
+        <v>0.55019015312911712</v>
       </c>
       <c r="H37" s="12">
-        <v>1.532998388181952E-2</v>
+        <v>0.62756353499656081</v>
       </c>
       <c r="I37" s="12">
-        <v>0.29408265831335001</v>
+        <v>1.9264605376319219</v>
       </c>
       <c r="J37" s="12">
-        <v>0.1097603211429076</v>
+        <v>9.8541326104743202E-3</v>
       </c>
       <c r="K37" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L37" s="10" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="M37" s="7"/>
       <c r="N37" s="7"/>
@@ -4681,13 +4672,11 @@
         <v>23</v>
       </c>
       <c r="R37" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="S37" s="2" t="s">
-        <v>61</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="S37" s="2"/>
       <c r="T37" s="2" t="s">
-        <v>62</v>
+        <v>95</v>
       </c>
       <c r="U37" s="2"/>
       <c r="V37" s="2" t="s">
@@ -4697,13 +4686,13 @@
         <v>23</v>
       </c>
       <c r="X37" s="2">
-        <v>164.0718</v>
+        <v>262.06950000000001</v>
       </c>
       <c r="Y37" s="2">
-        <v>58</v>
+        <v>134</v>
       </c>
       <c r="Z37" s="2" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="AA37" s="2" t="s">
         <v>29</v>
@@ -4716,42 +4705,48 @@
     </row>
     <row r="38" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>165</v>
+        <v>36</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C38" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="G38" s="12">
-        <v>0.31242018585406578</v>
+        <v>0.41550808127715649</v>
       </c>
       <c r="H38" s="12">
-        <v>3.34157587829343E-3</v>
+        <v>0.42507349571591369</v>
       </c>
       <c r="I38" s="12">
-        <v>4.794351271877062E-2</v>
+        <v>1.256760204695194</v>
       </c>
       <c r="J38" s="12">
-        <v>0.78408739378422754</v>
+        <v>4.4252755026857682E-3</v>
       </c>
       <c r="K38" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L38" s="10" t="s">
-        <v>335</v>
-      </c>
-      <c r="M38" s="7"/>
-      <c r="N38" s="7"/>
-      <c r="O38" s="7"/>
+        <v>304</v>
+      </c>
+      <c r="M38" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N38" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="O38" s="7" t="s">
+        <v>24</v>
+      </c>
       <c r="P38" s="5" t="s">
         <v>23</v>
       </c>
@@ -4759,13 +4754,13 @@
         <v>23</v>
       </c>
       <c r="R38" s="2" t="s">
-        <v>166</v>
+        <v>37</v>
       </c>
       <c r="S38" s="2" t="s">
-        <v>167</v>
+        <v>38</v>
       </c>
       <c r="T38" s="2" t="s">
-        <v>168</v>
+        <v>39</v>
       </c>
       <c r="U38" s="2"/>
       <c r="V38" s="2" t="s">
@@ -4775,13 +4770,13 @@
         <v>23</v>
       </c>
       <c r="X38" s="2">
-        <v>165.05459999999999</v>
+        <v>89.024500000000003</v>
       </c>
       <c r="Y38" s="2">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="Z38" s="2" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="AA38" s="2" t="s">
         <v>29</v>
@@ -4794,38 +4789,38 @@
     </row>
     <row r="39" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>83</v>
+        <v>206</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="C39" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D39" s="2"/>
       <c r="E39" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>355</v>
+        <v>369</v>
       </c>
       <c r="G39" s="12">
-        <v>0.74213009626279813</v>
+        <v>0.81129313979982598</v>
       </c>
       <c r="H39" s="12">
-        <v>7.0743312657492357E-3</v>
+        <v>0.39017026025005369</v>
       </c>
       <c r="I39" s="12">
-        <v>-0.20339225141119319</v>
+        <v>1.4308769326288799</v>
       </c>
       <c r="J39" s="12">
-        <v>0.65523178463825249</v>
+        <v>4.0284930069031888E-2</v>
       </c>
       <c r="K39" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L39" s="10" t="s">
-        <v>314</v>
+        <v>345</v>
       </c>
       <c r="M39" s="7"/>
       <c r="N39" s="7"/>
@@ -4837,11 +4832,11 @@
         <v>23</v>
       </c>
       <c r="R39" s="2" t="s">
-        <v>84</v>
+        <v>207</v>
       </c>
       <c r="S39" s="2"/>
       <c r="T39" s="2" t="s">
-        <v>85</v>
+        <v>208</v>
       </c>
       <c r="U39" s="2"/>
       <c r="V39" s="2" t="s">
@@ -4851,13 +4846,13 @@
         <v>23</v>
       </c>
       <c r="X39" s="2">
-        <v>229.01230000000001</v>
+        <v>283.14440000000002</v>
       </c>
       <c r="Y39" s="2">
-        <v>199</v>
+        <v>51</v>
       </c>
       <c r="Z39" s="2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="AA39" s="2" t="s">
         <v>29</v>
@@ -4870,38 +4865,38 @@
     </row>
     <row r="40" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="C40" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="G40" s="12">
-        <v>0.58223576143027067</v>
+        <v>0.26808666413641552</v>
       </c>
       <c r="H40" s="12">
-        <v>4.2694027106335783E-2</v>
+        <v>0.1217336748932811</v>
       </c>
       <c r="I40" s="12">
-        <v>0.39619576717556088</v>
+        <v>0.58286136999222293</v>
       </c>
       <c r="J40" s="12">
-        <v>0.28127257421310192</v>
+        <v>1.042644163461523E-2</v>
       </c>
       <c r="K40" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L40" s="10" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="M40" s="7"/>
       <c r="N40" s="7"/>
@@ -4913,13 +4908,13 @@
         <v>23</v>
       </c>
       <c r="R40" s="2" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="S40" s="2" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="T40" s="2" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="U40" s="2"/>
       <c r="V40" s="2" t="s">
@@ -4929,13 +4924,13 @@
         <v>23</v>
       </c>
       <c r="X40" s="2">
-        <v>379.03930000000003</v>
+        <v>123.0552</v>
       </c>
       <c r="Y40" s="2">
-        <v>147</v>
+        <v>27</v>
       </c>
       <c r="Z40" s="2" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="AA40" s="2" t="s">
         <v>29</v>
@@ -4948,38 +4943,38 @@
     </row>
     <row r="41" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>71</v>
+        <v>221</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>376</v>
+        <v>221</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="G41" s="12">
-        <v>0.40997998758135168</v>
+        <v>-0.33965849253399227</v>
       </c>
       <c r="H41" s="12">
-        <v>5.8644107209904336E-3</v>
+        <v>3.6618152455387382E-2</v>
       </c>
       <c r="I41" s="12">
-        <v>0.27764180048433929</v>
+        <v>-4.0004918219270991E-2</v>
       </c>
       <c r="J41" s="12">
-        <v>0.26137876946803812</v>
+        <v>0.87143115416330019</v>
       </c>
       <c r="K41" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L41" s="10" t="s">
-        <v>312</v>
+        <v>347</v>
       </c>
       <c r="M41" s="7"/>
       <c r="N41" s="7"/>
@@ -4991,13 +4986,11 @@
         <v>23</v>
       </c>
       <c r="R41" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="S41" s="2" t="s">
-        <v>73</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="S41" s="2"/>
       <c r="T41" s="2" t="s">
-        <v>74</v>
+        <v>223</v>
       </c>
       <c r="U41" s="2"/>
       <c r="V41" s="2" t="s">
@@ -5007,16 +5000,16 @@
         <v>23</v>
       </c>
       <c r="X41" s="2">
-        <v>180.06659999999999</v>
+        <v>336.05275999999998</v>
       </c>
       <c r="Y41" s="2">
-        <v>58</v>
+        <v>154.60715999999999</v>
       </c>
       <c r="Z41" s="2" t="s">
-        <v>35</v>
+        <v>224</v>
       </c>
       <c r="AA41" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AB41" s="2" t="s">
         <v>23</v>
@@ -5026,38 +5019,38 @@
     </row>
     <row r="42" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>131</v>
+        <v>198</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D42" s="2"/>
-      <c r="E42" s="2" t="s">
+      <c r="E42" s="11" t="s">
         <v>399</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="G42" s="12">
-        <v>0.78621412149081848</v>
+        <v>0.78788027038367225</v>
       </c>
       <c r="H42" s="12">
-        <v>1.3185947511990931E-2</v>
+        <v>1.214756412959191E-2</v>
       </c>
       <c r="I42" s="12">
-        <v>0.28763142206793191</v>
+        <v>1.09017017963679</v>
       </c>
       <c r="J42" s="12">
-        <v>0.43716304463804939</v>
+        <v>1.8861574903656489E-2</v>
       </c>
       <c r="K42" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L42" s="10" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
       <c r="M42" s="7"/>
       <c r="N42" s="7"/>
@@ -5069,11 +5062,11 @@
         <v>23</v>
       </c>
       <c r="R42" s="2" t="s">
-        <v>132</v>
+        <v>199</v>
       </c>
       <c r="S42" s="2"/>
       <c r="T42" s="2" t="s">
-        <v>133</v>
+        <v>205</v>
       </c>
       <c r="U42" s="2"/>
       <c r="V42" s="2" t="s">
@@ -5083,16 +5076,16 @@
         <v>23</v>
       </c>
       <c r="X42" s="2">
-        <v>398.00619999999998</v>
+        <v>263.11142000000001</v>
       </c>
       <c r="Y42" s="2">
-        <v>138</v>
+        <v>200.12349</v>
       </c>
       <c r="Z42" s="2" t="s">
-        <v>40</v>
+        <v>142</v>
       </c>
       <c r="AA42" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AB42" s="2" t="s">
         <v>23</v>
@@ -5102,10 +5095,10 @@
     </row>
     <row r="43" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>386</v>
+        <v>172</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>24</v>
@@ -5115,25 +5108,25 @@
         <v>399</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="G43" s="12">
-        <v>0.53781869393490922</v>
+        <v>1.9866722893218101</v>
       </c>
       <c r="H43" s="12">
-        <v>3.7055885051282877E-2</v>
+        <v>3.6670247228030292E-2</v>
       </c>
       <c r="I43" s="12">
-        <v>0.13663548694990621</v>
+        <v>1.062516150760739</v>
       </c>
       <c r="J43" s="12">
-        <v>0.55005347203021426</v>
+        <v>0.24272368503491659</v>
       </c>
       <c r="K43" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L43" s="10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="M43" s="7"/>
       <c r="N43" s="7"/>
@@ -5145,13 +5138,11 @@
         <v>23</v>
       </c>
       <c r="R43" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="S43" s="2" t="s">
-        <v>180</v>
-      </c>
+        <v>173</v>
+      </c>
+      <c r="S43" s="2"/>
       <c r="T43" s="2" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="U43" s="2"/>
       <c r="V43" s="2" t="s">
@@ -5161,16 +5152,16 @@
         <v>23</v>
       </c>
       <c r="X43" s="2">
-        <v>198.0881</v>
+        <v>191.092198</v>
       </c>
       <c r="Y43" s="2">
-        <v>59</v>
+        <v>48.571967999999998</v>
       </c>
       <c r="Z43" s="2" t="s">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="AA43" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AB43" s="2" t="s">
         <v>23</v>
@@ -5180,10 +5171,10 @@
     </row>
     <row r="44" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>225</v>
+        <v>67</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>24</v>
@@ -5193,25 +5184,25 @@
         <v>399</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="G44" s="12">
-        <v>1.449497195603316</v>
+        <v>-0.10961756670894469</v>
       </c>
       <c r="H44" s="12">
-        <v>2.4084407570208119E-3</v>
+        <v>2.257269706394751E-2</v>
       </c>
       <c r="I44" s="12">
-        <v>0.52907850064326922</v>
+        <v>-7.9505608410148199E-2</v>
       </c>
       <c r="J44" s="12">
-        <v>0.36733938692032359</v>
+        <v>0.46920552554535561</v>
       </c>
       <c r="K44" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L44" s="10" t="s">
-        <v>348</v>
+        <v>311</v>
       </c>
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
@@ -5223,11 +5214,13 @@
         <v>23</v>
       </c>
       <c r="R44" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="S44" s="2"/>
+        <v>68</v>
+      </c>
+      <c r="S44" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="T44" s="2" t="s">
-        <v>227</v>
+        <v>70</v>
       </c>
       <c r="U44" s="2"/>
       <c r="V44" s="2" t="s">
@@ -5237,16 +5230,16 @@
         <v>23</v>
       </c>
       <c r="X44" s="2">
-        <v>339.17747600000001</v>
+        <v>180.0335</v>
       </c>
       <c r="Y44" s="2">
-        <v>204.30355800000001</v>
+        <v>130</v>
       </c>
       <c r="Z44" s="2" t="s">
-        <v>228</v>
+        <v>40</v>
       </c>
       <c r="AA44" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AB44" s="2" t="s">
         <v>23</v>
@@ -5256,38 +5249,38 @@
     </row>
     <row r="45" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>221</v>
+        <v>384</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="G45" s="12">
-        <v>-0.33965849253399227</v>
+        <v>1.779746875546653</v>
       </c>
       <c r="H45" s="12">
-        <v>3.6618152455387382E-2</v>
+        <v>3.4638840419138168E-5</v>
       </c>
       <c r="I45" s="12">
-        <v>-4.0004918219270991E-2</v>
+        <v>-0.47542374833514067</v>
       </c>
       <c r="J45" s="12">
-        <v>0.87143115416330019</v>
+        <v>0.63892167026263857</v>
       </c>
       <c r="K45" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L45" s="10" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="M45" s="7"/>
       <c r="N45" s="7"/>
@@ -5299,11 +5292,13 @@
         <v>23</v>
       </c>
       <c r="R45" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="S45" s="2"/>
+        <v>218</v>
+      </c>
+      <c r="S45" s="2" t="s">
+        <v>219</v>
+      </c>
       <c r="T45" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="U45" s="2"/>
       <c r="V45" s="2" t="s">
@@ -5313,16 +5308,16 @@
         <v>23</v>
       </c>
       <c r="X45" s="2">
-        <v>336.05275999999998</v>
+        <v>335.09500000000003</v>
       </c>
       <c r="Y45" s="2">
-        <v>154.60715999999999</v>
+        <v>183</v>
       </c>
       <c r="Z45" s="2" t="s">
-        <v>224</v>
+        <v>141</v>
       </c>
       <c r="AA45" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AB45" s="2" t="s">
         <v>23</v>
@@ -5332,54 +5327,56 @@
     </row>
     <row r="46" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>198</v>
+        <v>89</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>378</v>
+        <v>89</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D46" s="2"/>
-      <c r="E46" s="11" t="s">
-        <v>400</v>
+      <c r="E46" s="2" t="s">
+        <v>421</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="G46" s="12">
-        <v>0.78788027038367225</v>
+        <v>-0.21232771886722551</v>
       </c>
       <c r="H46" s="12">
-        <v>1.214756412959191E-2</v>
+        <v>3.2347958530699238E-2</v>
       </c>
       <c r="I46" s="12">
-        <v>1.09017017963679</v>
+        <v>6.2649205201758207E-2</v>
       </c>
       <c r="J46" s="12">
-        <v>1.8861574903656489E-2</v>
+        <v>0.56166950064806109</v>
       </c>
       <c r="K46" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L46" s="10" t="s">
-        <v>343</v>
+        <v>315</v>
       </c>
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
       <c r="O46" s="7"/>
       <c r="P46" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q46" s="5" t="s">
         <v>23</v>
       </c>
       <c r="R46" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="S46" s="2"/>
+        <v>90</v>
+      </c>
+      <c r="S46" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="T46" s="2" t="s">
-        <v>205</v>
+        <v>92</v>
       </c>
       <c r="U46" s="2"/>
       <c r="V46" s="2" t="s">
@@ -5389,16 +5386,16 @@
         <v>23</v>
       </c>
       <c r="X46" s="2">
-        <v>263.11142000000001</v>
+        <v>242.06989999999999</v>
       </c>
       <c r="Y46" s="2">
-        <v>200.12349</v>
+        <v>148</v>
       </c>
       <c r="Z46" s="2" t="s">
-        <v>142</v>
+        <v>40</v>
       </c>
       <c r="AA46" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AB46" s="2" t="s">
         <v>23</v>
@@ -5408,38 +5405,38 @@
     </row>
     <row r="47" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>172</v>
+        <v>134</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C47" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D47" s="2"/>
       <c r="E47" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>357</v>
+        <v>421</v>
+      </c>
+      <c r="F47" s="11" t="s">
+        <v>361</v>
       </c>
       <c r="G47" s="12">
-        <v>1.9866722893218101</v>
+        <v>0.24141717347866631</v>
       </c>
       <c r="H47" s="12">
-        <v>3.6670247228030292E-2</v>
+        <v>0.55280427491186623</v>
       </c>
       <c r="I47" s="12">
-        <v>1.062516150760739</v>
+        <v>2.0707014376494581</v>
       </c>
       <c r="J47" s="12">
-        <v>0.24272368503491659</v>
+        <v>1.7532161293423039E-3</v>
       </c>
       <c r="K47" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L47" s="10" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
@@ -5451,11 +5448,11 @@
         <v>23</v>
       </c>
       <c r="R47" s="2" t="s">
-        <v>173</v>
+        <v>135</v>
       </c>
       <c r="S47" s="2"/>
       <c r="T47" s="2" t="s">
-        <v>174</v>
+        <v>136</v>
       </c>
       <c r="U47" s="2"/>
       <c r="V47" s="2" t="s">
@@ -5465,13 +5462,13 @@
         <v>23</v>
       </c>
       <c r="X47" s="2">
-        <v>191.092198</v>
+        <v>407.20750099999998</v>
       </c>
       <c r="Y47" s="2">
-        <v>48.571967999999998</v>
+        <v>153.490116</v>
       </c>
       <c r="Z47" s="2" t="s">
-        <v>160</v>
+        <v>54</v>
       </c>
       <c r="AA47" s="2" t="s">
         <v>25</v>
@@ -5484,38 +5481,38 @@
     </row>
     <row r="48" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>67</v>
+        <v>115</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="C48" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D48" s="2"/>
       <c r="E48" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>369</v>
+        <v>421</v>
+      </c>
+      <c r="F48" s="11" t="s">
+        <v>361</v>
       </c>
       <c r="G48" s="12">
-        <v>-0.10961756670894469</v>
+        <v>0.52082421505483723</v>
       </c>
       <c r="H48" s="12">
-        <v>2.257269706394751E-2</v>
+        <v>0.18143830225368149</v>
       </c>
       <c r="I48" s="12">
-        <v>-7.9505608410148199E-2</v>
+        <v>1.2338926633816949</v>
       </c>
       <c r="J48" s="12">
-        <v>0.46920552554535561</v>
+        <v>2.0195633925086439E-3</v>
       </c>
       <c r="K48" s="8" t="s">
         <v>303</v>
       </c>
       <c r="L48" s="10" t="s">
-        <v>311</v>
+        <v>321</v>
       </c>
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
@@ -5527,13 +5524,13 @@
         <v>23</v>
       </c>
       <c r="R48" s="2" t="s">
-        <v>68</v>
+        <v>116</v>
       </c>
       <c r="S48" s="2" t="s">
-        <v>69</v>
+        <v>117</v>
       </c>
       <c r="T48" s="2" t="s">
-        <v>70</v>
+        <v>118</v>
       </c>
       <c r="U48" s="2"/>
       <c r="V48" s="2" t="s">
@@ -5543,13 +5540,13 @@
         <v>23</v>
       </c>
       <c r="X48" s="2">
-        <v>180.0335</v>
+        <v>367.15780000000001</v>
       </c>
       <c r="Y48" s="2">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="Z48" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="AA48" s="2" t="s">
         <v>29</v>
@@ -5648,7 +5645,7 @@
       </c>
       <c r="D50" s="2"/>
       <c r="E50" s="2" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>360</v>
@@ -5875,7 +5872,7 @@
         <v>235</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>24</v>
@@ -5949,7 +5946,11 @@
       <c r="AD53" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD53" xr:uid="{00D18420-3B44-BF43-B42B-A5B659E984D7}"/>
+  <autoFilter ref="A1:AD53" xr:uid="{00D18420-3B44-BF43-B42B-A5B659E984D7}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AD53">
+      <sortCondition ref="E1:E53"/>
+    </sortState>
+  </autoFilter>
   <conditionalFormatting sqref="H2:H53">
     <cfRule type="cellIs" dxfId="7" priority="3" operator="between">
       <formula>0.1</formula>
@@ -5993,22 +5994,22 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>247</v>
       </c>
       <c r="E1" s="13" t="s">
+        <v>403</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>404</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>405</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>396</v>
@@ -6035,7 +6036,7 @@
         <v>209</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E2" s="2">
         <v>0.256162021422708</v>
@@ -6158,7 +6159,7 @@
         <v>290</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>289</v>
@@ -6173,7 +6174,7 @@
         <v>398</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>248</v>
@@ -6249,7 +6250,7 @@
         <v>44</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E9" s="2">
         <v>0.322021181136739</v>
@@ -6291,7 +6292,7 @@
         <v>398</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>262</v>
@@ -6405,7 +6406,7 @@
         <v>252</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E14" s="2">
         <v>1.01356036325546</v>
@@ -6437,7 +6438,7 @@
         <v>295</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E15" s="2">
         <v>1.82124944684701</v>
@@ -6497,7 +6498,7 @@
         <v>286</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="E17" s="2">
         <v>-1.3004528435882801</v>
@@ -6509,7 +6510,7 @@
         <v>398</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>287</v>
@@ -6527,7 +6528,7 @@
         <v>279</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E18" s="2">
         <v>1.1563624217516999</v>
@@ -6539,7 +6540,7 @@
         <v>398</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>280</v>
@@ -6571,7 +6572,7 @@
         <v>398</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>276</v>
@@ -6600,7 +6601,7 @@
         <v>4.5434876280894702E-2</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>399</v>
+        <v>421</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>364</v>
@@ -6630,10 +6631,10 @@
         <v>4.9199430497781402E-2</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>399</v>
+        <v>421</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>284</v>
@@ -6660,7 +6661,7 @@
         <v>1.03135448211868E-2</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>399</v>
+        <v>421</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>355</v>
@@ -6689,7 +6690,7 @@
       <c r="F23" s="14">
         <v>2.5261982283094099E-2</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="G23" s="2" t="s">
         <v>421</v>
       </c>
       <c r="H23" s="2" t="s">
@@ -6713,7 +6714,7 @@
         <v>269</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E24" s="2">
         <v>1.4230672997023699</v>
@@ -6721,7 +6722,7 @@
       <c r="F24" s="14">
         <v>1.7590258420630101E-2</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="2" t="s">
         <v>421</v>
       </c>
       <c r="H24" s="2" t="s">
@@ -6743,7 +6744,7 @@
         <v>272</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E25" s="2">
         <v>0.44088254428074403</v>
@@ -6751,7 +6752,7 @@
       <c r="F25" s="14">
         <v>3.5150109902689201E-3</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="G25" s="2" t="s">
         <v>421</v>
       </c>
       <c r="H25" s="2" t="s">
@@ -6781,11 +6782,11 @@
       <c r="F26" s="14">
         <v>3.8536356428932099E-2</v>
       </c>
-      <c r="G26" s="11" t="s">
-        <v>421</v>
+      <c r="G26" s="2" t="s">
+        <v>398</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>218</v>
@@ -6813,7 +6814,7 @@
       <c r="F27" s="14">
         <v>3.4181998392058703E-2</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G27" s="2" t="s">
         <v>421</v>
       </c>
       <c r="H27" s="2" t="s">
@@ -6849,40 +6850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Resident xmlns="2b2e4ec7-6b51-40d9-a657-413b8d106af2">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Resident>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2b2e4ec7-6b51-40d9-a657-413b8d106af2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="12e8c7ec-5f59-40ef-b1ca-d288221f299b" xsi:nil="true"/>
-    <Assignment xmlns="2b2e4ec7-6b51-40d9-a657-413b8d106af2">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Assignment>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A53F7F2A09069342814081195BEB0A4C" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7664040cc87d199f5d7d596277ddc936">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2b2e4ec7-6b51-40d9-a657-413b8d106af2" xmlns:ns3="12e8c7ec-5f59-40ef-b1ca-d288221f299b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cd2af0efcefca0176de1c9ac0642644f" ns2:_="" ns3:_="">
     <xsd:import namespace="2b2e4ec7-6b51-40d9-a657-413b8d106af2"/>
@@ -7157,10 +7124,55 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Resident xmlns="2b2e4ec7-6b51-40d9-a657-413b8d106af2">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Resident>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2b2e4ec7-6b51-40d9-a657-413b8d106af2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="12e8c7ec-5f59-40ef-b1ca-d288221f299b" xsi:nil="true"/>
+    <Assignment xmlns="2b2e4ec7-6b51-40d9-a657-413b8d106af2">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Assignment>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FA52A0C-9929-4B5E-9232-E7068BC31D29}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3064440-F24A-45C7-8114-8B1E938CC9C3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2b2e4ec7-6b51-40d9-a657-413b8d106af2"/>
+    <ds:schemaRef ds:uri="12e8c7ec-5f59-40ef-b1ca-d288221f299b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7183,20 +7195,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3064440-F24A-45C7-8114-8B1E938CC9C3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FA52A0C-9929-4B5E-9232-E7068BC31D29}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2b2e4ec7-6b51-40d9-a657-413b8d106af2"/>
-    <ds:schemaRef ds:uri="12e8c7ec-5f59-40ef-b1ca-d288221f299b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
did big figure update- added AMP figure in fig 4
</commit_message>
<xml_diff>
--- a/Databases/QC/manual_QC_repo.xlsx
+++ b/Databases/QC/manual_QC_repo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11209"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdp2019/Desktop/PGD-postop-metabolomics/Databases/QC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/JoshsMacbook2015/Desktop/PGD-postop-metabolomics/Databases/QC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E5EA3A-C2C0-7D43-9E43-557915946659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27CEFFC-3F76-ED48-82A0-6C4C48F456D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="22560" windowHeight="17720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="38400" windowHeight="20840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="curated_spec" sheetId="16" r:id="rId1"/>
@@ -1388,7 +1388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1420,6 +1420,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5985,7 +5986,7 @@
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="44.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -6038,7 +6039,7 @@
       <c r="D2" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="15">
         <v>0.256162021422708</v>
       </c>
       <c r="F2" s="14">
@@ -6070,7 +6071,7 @@
       <c r="D3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="15">
         <v>1.1418062428519</v>
       </c>
       <c r="F3" s="14">
@@ -6102,7 +6103,7 @@
       <c r="D4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="15">
         <v>-1.77812695212567</v>
       </c>
       <c r="F4" s="14">
@@ -6132,7 +6133,7 @@
       <c r="D5" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="15">
         <v>0.49466166232049802</v>
       </c>
       <c r="F5" s="14">
@@ -6164,7 +6165,7 @@
       <c r="D6" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="15">
         <v>0.92440004113679297</v>
       </c>
       <c r="F6" s="14">
@@ -6194,7 +6195,7 @@
       <c r="D7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="15">
         <v>1.23559856307712</v>
       </c>
       <c r="F7" s="14">
@@ -6222,7 +6223,7 @@
       <c r="D8" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="15">
         <v>0.39363163110403498</v>
       </c>
       <c r="F8" s="14">
@@ -6252,7 +6253,7 @@
       <c r="D9" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="15">
         <v>0.322021181136739</v>
       </c>
       <c r="F9" s="14">
@@ -6282,7 +6283,7 @@
       <c r="D10" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="15">
         <v>0.93867167998641299</v>
       </c>
       <c r="F10" s="14">
@@ -6314,7 +6315,7 @@
       <c r="D11" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="15">
         <v>4.27245716629045</v>
       </c>
       <c r="F11" s="14">
@@ -6346,7 +6347,7 @@
       <c r="D12" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="15">
         <v>-2.1998505866778002</v>
       </c>
       <c r="F12" s="14">
@@ -6376,7 +6377,7 @@
       <c r="D13" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="15">
         <v>0.93309931204943497</v>
       </c>
       <c r="F13" s="14">
@@ -6408,7 +6409,7 @@
       <c r="D14" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="15">
         <v>1.01356036325546</v>
       </c>
       <c r="F14" s="14">
@@ -6440,7 +6441,7 @@
       <c r="D15" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="15">
         <v>1.82124944684701</v>
       </c>
       <c r="F15" s="14">
@@ -6470,7 +6471,7 @@
       <c r="D16" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="15">
         <v>2.6465198855318199</v>
       </c>
       <c r="F16" s="14">
@@ -6500,7 +6501,7 @@
       <c r="D17" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="15">
         <v>-1.3004528435882801</v>
       </c>
       <c r="F17" s="14">
@@ -6530,7 +6531,7 @@
       <c r="D18" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="15">
         <v>1.1563624217516999</v>
       </c>
       <c r="F18" s="14">
@@ -6562,7 +6563,7 @@
       <c r="D19" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="15">
         <v>1.3925592065805501</v>
       </c>
       <c r="F19" s="14">
@@ -6594,7 +6595,7 @@
       <c r="D20" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="15">
         <v>2.18569023810698</v>
       </c>
       <c r="F20" s="14">
@@ -6624,7 +6625,7 @@
       <c r="D21" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="15">
         <v>-1.6291493654188101</v>
       </c>
       <c r="F21" s="14">
@@ -6654,7 +6655,7 @@
       <c r="D22" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="15">
         <v>1.2779529723504801</v>
       </c>
       <c r="F22" s="14">
@@ -6684,7 +6685,7 @@
       <c r="D23" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="15">
         <v>0.27494757800842301</v>
       </c>
       <c r="F23" s="14">
@@ -6716,7 +6717,7 @@
       <c r="D24" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="15">
         <v>1.4230672997023699</v>
       </c>
       <c r="F24" s="14">
@@ -6746,7 +6747,7 @@
       <c r="D25" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="15">
         <v>0.44088254428074403</v>
       </c>
       <c r="F25" s="14">
@@ -6776,7 +6777,7 @@
       <c r="D26" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="15">
         <v>-2.2508408670334399</v>
       </c>
       <c r="F26" s="14">
@@ -6808,7 +6809,7 @@
       <c r="D27" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="15">
         <v>1.82007337011589</v>
       </c>
       <c r="F27" s="14">
@@ -6850,6 +6851,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A53F7F2A09069342814081195BEB0A4C" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7664040cc87d199f5d7d596277ddc936">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2b2e4ec7-6b51-40d9-a657-413b8d106af2" xmlns:ns3="12e8c7ec-5f59-40ef-b1ca-d288221f299b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cd2af0efcefca0176de1c9ac0642644f" ns2:_="" ns3:_="">
     <xsd:import namespace="2b2e4ec7-6b51-40d9-a657-413b8d106af2"/>
@@ -7124,7 +7134,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Resident xmlns="2b2e4ec7-6b51-40d9-a657-413b8d106af2">
@@ -7149,16 +7159,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FA52A0C-9929-4B5E-9232-E7068BC31D29}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3064440-F24A-45C7-8114-8B1E938CC9C3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7177,7 +7186,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AEC97AB-2352-42BA-9A7F-AB3618733AEC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -7192,12 +7201,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FA52A0C-9929-4B5E-9232-E7068BC31D29}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>